<commit_message>
Corrected the Metadata worksheet in the example xlsx files so that the version is 4.1, not 4
</commit_message>
<xml_diff>
--- a/doc/_static/example-files/PMHC-4-1-combined-delete.xlsx
+++ b/doc/_static/example-files/PMHC-4-1-combined-delete.xlsx
@@ -1,10 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10413"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jennib/Work/git/PMHC/spec/doc/_static/example-files/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{85F30D1D-0AA7-6145-A94C-382C0F9A0867}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView xWindow="240" yWindow="760" windowWidth="16100" windowHeight="9660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Metadata" sheetId="1" r:id="rId1"/>
@@ -22,7 +28,7 @@
     <sheet name="Service Contact Practitioners" sheetId="13" r:id="rId13"/>
     <sheet name="Practitioners" sheetId="14" r:id="rId14"/>
   </sheets>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519"/>
 </workbook>
 </file>
 
@@ -959,8 +965,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -997,13 +1003,21 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1041,7 +1055,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -1075,6 +1089,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -1109,9 +1124,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1284,11 +1300,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B3"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1296,7 +1312,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -1304,12 +1320,12 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:2">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>4</v>
       </c>
       <c r="B3">
-        <v>4</v>
+        <v>4.0999999999999996</v>
       </c>
     </row>
   </sheetData>
@@ -1318,11 +1334,11 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
   <dimension ref="A1:K11"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:11">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>5</v>
       </c>
@@ -1357,7 +1373,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="2" spans="1:11">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>16</v>
       </c>
@@ -1368,7 +1384,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:11">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>16</v>
       </c>
@@ -1379,7 +1395,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="4" spans="1:11">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>16</v>
       </c>
@@ -1390,7 +1406,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="5" spans="1:11">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>16</v>
       </c>
@@ -1401,7 +1417,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:11">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>16</v>
       </c>
@@ -1412,7 +1428,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="7" spans="1:11">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>16</v>
       </c>
@@ -1423,7 +1439,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="8" spans="1:11">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>16</v>
       </c>
@@ -1434,7 +1450,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="9" spans="1:11">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>16</v>
       </c>
@@ -1445,7 +1461,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="10" spans="1:11">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>16</v>
       </c>
@@ -1456,7 +1472,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="11" spans="1:11">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>16</v>
       </c>
@@ -1473,11 +1489,11 @@
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
   <dimension ref="A1:BC22"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:55">
+    <row r="1" spans="1:55" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>5</v>
       </c>
@@ -1644,7 +1660,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="2" spans="1:55">
+    <row r="2" spans="1:55" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>16</v>
       </c>
@@ -1655,7 +1671,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:55">
+    <row r="3" spans="1:55" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>16</v>
       </c>
@@ -1666,7 +1682,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="4" spans="1:55">
+    <row r="4" spans="1:55" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>16</v>
       </c>
@@ -1677,7 +1693,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="5" spans="1:55">
+    <row r="5" spans="1:55" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>16</v>
       </c>
@@ -1688,7 +1704,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:55">
+    <row r="6" spans="1:55" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>16</v>
       </c>
@@ -1699,7 +1715,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="7" spans="1:55">
+    <row r="7" spans="1:55" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>16</v>
       </c>
@@ -1710,7 +1726,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="8" spans="1:55">
+    <row r="8" spans="1:55" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>16</v>
       </c>
@@ -1721,7 +1737,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="9" spans="1:55">
+    <row r="9" spans="1:55" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>16</v>
       </c>
@@ -1732,7 +1748,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="10" spans="1:55">
+    <row r="10" spans="1:55" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>16</v>
       </c>
@@ -1743,7 +1759,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="11" spans="1:55">
+    <row r="11" spans="1:55" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>16</v>
       </c>
@@ -1754,7 +1770,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="12" spans="1:55">
+    <row r="12" spans="1:55" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>16</v>
       </c>
@@ -1765,7 +1781,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="13" spans="1:55">
+    <row r="13" spans="1:55" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>16</v>
       </c>
@@ -1776,7 +1792,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="14" spans="1:55">
+    <row r="14" spans="1:55" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>16</v>
       </c>
@@ -1787,7 +1803,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="15" spans="1:55">
+    <row r="15" spans="1:55" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>16</v>
       </c>
@@ -1798,7 +1814,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="16" spans="1:55">
+    <row r="16" spans="1:55" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>16</v>
       </c>
@@ -1809,7 +1825,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="17" spans="1:3">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>16</v>
       </c>
@@ -1820,7 +1836,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="18" spans="1:3">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>16</v>
       </c>
@@ -1831,7 +1847,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="19" spans="1:3">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>16</v>
       </c>
@@ -1842,7 +1858,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="20" spans="1:3">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>16</v>
       </c>
@@ -1853,7 +1869,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="21" spans="1:3">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>16</v>
       </c>
@@ -1864,7 +1880,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="22" spans="1:3">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>16</v>
       </c>
@@ -1881,11 +1897,11 @@
 </file>
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0B00-000000000000}">
   <dimension ref="A1:T11"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:20">
+    <row r="1" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>5</v>
       </c>
@@ -1947,7 +1963,7 @@
         <v>266</v>
       </c>
     </row>
-    <row r="2" spans="1:20">
+    <row r="2" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>16</v>
       </c>
@@ -1958,7 +1974,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:20">
+    <row r="3" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>16</v>
       </c>
@@ -1969,7 +1985,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="4" spans="1:20">
+    <row r="4" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>16</v>
       </c>
@@ -1980,7 +1996,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="5" spans="1:20">
+    <row r="5" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>16</v>
       </c>
@@ -1991,7 +2007,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:20">
+    <row r="6" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>16</v>
       </c>
@@ -2002,7 +2018,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="7" spans="1:20">
+    <row r="7" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>16</v>
       </c>
@@ -2013,7 +2029,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="8" spans="1:20">
+    <row r="8" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>16</v>
       </c>
@@ -2024,7 +2040,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="9" spans="1:20">
+    <row r="9" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>16</v>
       </c>
@@ -2035,7 +2051,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="10" spans="1:20">
+    <row r="10" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>16</v>
       </c>
@@ -2046,7 +2062,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="11" spans="1:20">
+    <row r="11" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>16</v>
       </c>
@@ -2063,11 +2079,11 @@
 </file>
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0C00-000000000000}">
   <dimension ref="A1:F13"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>5</v>
       </c>
@@ -2087,7 +2103,7 @@
         <v>279</v>
       </c>
     </row>
-    <row r="2" spans="1:6">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>16</v>
       </c>
@@ -2098,7 +2114,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:6">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>16</v>
       </c>
@@ -2109,7 +2125,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="4" spans="1:6">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>16</v>
       </c>
@@ -2120,7 +2136,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="5" spans="1:6">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>16</v>
       </c>
@@ -2131,7 +2147,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:6">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>16</v>
       </c>
@@ -2142,7 +2158,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="7" spans="1:6">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>16</v>
       </c>
@@ -2153,7 +2169,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="8" spans="1:6">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>16</v>
       </c>
@@ -2164,7 +2180,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="9" spans="1:6">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>16</v>
       </c>
@@ -2175,7 +2191,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="10" spans="1:6">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>16</v>
       </c>
@@ -2186,7 +2202,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="11" spans="1:6">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>16</v>
       </c>
@@ -2197,7 +2213,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="12" spans="1:6">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>16</v>
       </c>
@@ -2208,7 +2224,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="13" spans="1:6">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>16</v>
       </c>
@@ -2225,11 +2241,11 @@
 </file>
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0D00-000000000000}">
   <dimension ref="A1:J11"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:10">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>5</v>
       </c>
@@ -2261,7 +2277,7 @@
         <v>298</v>
       </c>
     </row>
-    <row r="2" spans="1:10">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>16</v>
       </c>
@@ -2272,7 +2288,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:10">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>16</v>
       </c>
@@ -2283,7 +2299,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="4" spans="1:10">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>16</v>
       </c>
@@ -2294,7 +2310,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="5" spans="1:10">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>16</v>
       </c>
@@ -2305,7 +2321,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:10">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>16</v>
       </c>
@@ -2316,7 +2332,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="7" spans="1:10">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>16</v>
       </c>
@@ -2327,7 +2343,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="8" spans="1:10">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>16</v>
       </c>
@@ -2338,7 +2354,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="9" spans="1:10">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>16</v>
       </c>
@@ -2349,7 +2365,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="10" spans="1:10">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>16</v>
       </c>
@@ -2360,7 +2376,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="11" spans="1:10">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>16</v>
       </c>
@@ -2377,11 +2393,11 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:K2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:11">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>5</v>
       </c>
@@ -2416,7 +2432,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="2" spans="1:11">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>16</v>
       </c>
@@ -2451,11 +2467,11 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:L6"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:12">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>5</v>
       </c>
@@ -2493,7 +2509,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="2" spans="1:12">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>16</v>
       </c>
@@ -2504,7 +2520,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:12">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>16</v>
       </c>
@@ -2515,7 +2531,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="4" spans="1:12">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>16</v>
       </c>
@@ -2526,7 +2542,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="5" spans="1:12">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>16</v>
       </c>
@@ -2537,7 +2553,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:12">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>16</v>
       </c>
@@ -2554,11 +2570,11 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:O11"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:15">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>5</v>
       </c>
@@ -2605,7 +2621,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="2" spans="1:15">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>16</v>
       </c>
@@ -2616,7 +2632,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:15">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>16</v>
       </c>
@@ -2627,7 +2643,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="4" spans="1:15">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>16</v>
       </c>
@@ -2638,7 +2654,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="5" spans="1:15">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>16</v>
       </c>
@@ -2649,7 +2665,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:15">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>16</v>
       </c>
@@ -2660,7 +2676,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="7" spans="1:15">
+    <row r="7" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>16</v>
       </c>
@@ -2671,7 +2687,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="8" spans="1:15">
+    <row r="8" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>16</v>
       </c>
@@ -2682,7 +2698,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="9" spans="1:15">
+    <row r="9" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>16</v>
       </c>
@@ -2693,7 +2709,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="10" spans="1:15">
+    <row r="10" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>16</v>
       </c>
@@ -2704,7 +2720,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="11" spans="1:15">
+    <row r="11" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>16</v>
       </c>
@@ -2721,11 +2737,11 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:P11"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:16">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>5</v>
       </c>
@@ -2775,7 +2791,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="2" spans="1:16">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>16</v>
       </c>
@@ -2786,7 +2802,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:16">
+    <row r="3" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>16</v>
       </c>
@@ -2797,7 +2813,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="4" spans="1:16">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>16</v>
       </c>
@@ -2808,7 +2824,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="5" spans="1:16">
+    <row r="5" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>16</v>
       </c>
@@ -2819,7 +2835,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:16">
+    <row r="6" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>16</v>
       </c>
@@ -2830,7 +2846,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="7" spans="1:16">
+    <row r="7" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>16</v>
       </c>
@@ -2841,7 +2857,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="8" spans="1:16">
+    <row r="8" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>16</v>
       </c>
@@ -2852,7 +2868,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="9" spans="1:16">
+    <row r="9" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>16</v>
       </c>
@@ -2863,7 +2879,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="10" spans="1:16">
+    <row r="10" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>16</v>
       </c>
@@ -2874,7 +2890,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="11" spans="1:16">
+    <row r="11" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>16</v>
       </c>
@@ -2891,11 +2907,11 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:AE11"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:31">
+    <row r="1" spans="1:31" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>5</v>
       </c>
@@ -2990,7 +3006,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="2" spans="1:31">
+    <row r="2" spans="1:31" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>16</v>
       </c>
@@ -3001,7 +3017,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:31">
+    <row r="3" spans="1:31" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>16</v>
       </c>
@@ -3012,7 +3028,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="4" spans="1:31">
+    <row r="4" spans="1:31" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>16</v>
       </c>
@@ -3023,7 +3039,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="5" spans="1:31">
+    <row r="5" spans="1:31" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>16</v>
       </c>
@@ -3034,7 +3050,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:31">
+    <row r="6" spans="1:31" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>16</v>
       </c>
@@ -3045,7 +3061,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="7" spans="1:31">
+    <row r="7" spans="1:31" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>16</v>
       </c>
@@ -3056,7 +3072,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="8" spans="1:31">
+    <row r="8" spans="1:31" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>16</v>
       </c>
@@ -3067,7 +3083,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="9" spans="1:31">
+    <row r="9" spans="1:31" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>16</v>
       </c>
@@ -3078,7 +3094,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="10" spans="1:31">
+    <row r="10" spans="1:31" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>16</v>
       </c>
@@ -3089,7 +3105,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="11" spans="1:31">
+    <row r="11" spans="1:31" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>16</v>
       </c>
@@ -3106,11 +3122,11 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:E11"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>113</v>
       </c>
@@ -3127,7 +3143,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="2" spans="1:5">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>16</v>
       </c>
@@ -3138,7 +3154,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:5">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>16</v>
       </c>
@@ -3149,7 +3165,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="4" spans="1:5">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>16</v>
       </c>
@@ -3160,7 +3176,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="5" spans="1:5">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>16</v>
       </c>
@@ -3171,7 +3187,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:5">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>16</v>
       </c>
@@ -3182,7 +3198,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="7" spans="1:5">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>16</v>
       </c>
@@ -3193,7 +3209,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="8" spans="1:5">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>16</v>
       </c>
@@ -3204,7 +3220,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="9" spans="1:5">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>16</v>
       </c>
@@ -3215,7 +3231,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="10" spans="1:5">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>16</v>
       </c>
@@ -3226,7 +3242,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="11" spans="1:5">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>16</v>
       </c>
@@ -3243,11 +3259,11 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1:G22"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:7">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>5</v>
       </c>
@@ -3270,7 +3286,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="2" spans="1:7">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>16</v>
       </c>
@@ -3281,7 +3297,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:7">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>16</v>
       </c>
@@ -3292,7 +3308,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="4" spans="1:7">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>16</v>
       </c>
@@ -3303,7 +3319,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="5" spans="1:7">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>16</v>
       </c>
@@ -3314,7 +3330,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:7">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>16</v>
       </c>
@@ -3325,7 +3341,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="7" spans="1:7">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>16</v>
       </c>
@@ -3336,7 +3352,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="8" spans="1:7">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>16</v>
       </c>
@@ -3347,7 +3363,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="9" spans="1:7">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>16</v>
       </c>
@@ -3358,7 +3374,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="10" spans="1:7">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>16</v>
       </c>
@@ -3369,7 +3385,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="11" spans="1:7">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>16</v>
       </c>
@@ -3380,7 +3396,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="12" spans="1:7">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>16</v>
       </c>
@@ -3391,7 +3407,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="13" spans="1:7">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>16</v>
       </c>
@@ -3402,7 +3418,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="14" spans="1:7">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>16</v>
       </c>
@@ -3413,7 +3429,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="15" spans="1:7">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>16</v>
       </c>
@@ -3424,7 +3440,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="16" spans="1:7">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>16</v>
       </c>
@@ -3435,7 +3451,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="17" spans="1:3">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>16</v>
       </c>
@@ -3446,7 +3462,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="18" spans="1:3">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>16</v>
       </c>
@@ -3457,7 +3473,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="19" spans="1:3">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>16</v>
       </c>
@@ -3468,7 +3484,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="20" spans="1:3">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>16</v>
       </c>
@@ -3479,7 +3495,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="21" spans="1:3">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>16</v>
       </c>
@@ -3490,7 +3506,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="22" spans="1:3">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>16</v>
       </c>
@@ -3507,11 +3523,11 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
   <dimension ref="A1:T6"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:20">
+    <row r="1" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>5</v>
       </c>
@@ -3573,7 +3589,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="2" spans="1:20">
+    <row r="2" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>16</v>
       </c>
@@ -3584,7 +3600,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:20">
+    <row r="3" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>16</v>
       </c>
@@ -3595,7 +3611,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="4" spans="1:20">
+    <row r="4" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>16</v>
       </c>
@@ -3606,7 +3622,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="5" spans="1:20">
+    <row r="5" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>16</v>
       </c>
@@ -3617,7 +3633,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:20">
+    <row r="6" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>16</v>
       </c>

</xml_diff>